<commit_message>
v1.0.0: Initial production release - ROI Calculator A-MAQ
</commit_message>
<xml_diff>
--- a/Calculadora_ROI_AMAQ.xlsx
+++ b/Calculadora_ROI_AMAQ.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9e70337b1991cbb/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\opencode\roicalculator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_5523B3152DF8ACBF09EF790670560CA704E1276F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2231DEC4-C382-4CC5-83BC-9B6AA59DEE73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -103,27 +103,18 @@
     <t>Características</t>
   </si>
   <si>
-    <t>Vidrio</t>
-  </si>
-  <si>
     <t>Básico</t>
   </si>
   <si>
     <t>Colector básico para rutas de inspección estándar</t>
   </si>
   <si>
-    <t>Ba 3 Pro</t>
-  </si>
-  <si>
     <t>Intermedio</t>
   </si>
   <si>
     <t>Colector profesional con análisis avanzado</t>
   </si>
   <si>
-    <t>Ba 5</t>
-  </si>
-  <si>
     <t>Full / Avanzado</t>
   </si>
   <si>
@@ -557,6 +548,15 @@
   </si>
   <si>
     <t>Fuentes: U.S. Department of Energy (DOE), McKinsey &amp; Company, PWC Predictive Maintenance 4.0, Metrix Vibration Methodology, Vista Projects ROI Guide</t>
+  </si>
+  <si>
+    <t>VibrioM</t>
+  </si>
+  <si>
+    <t>VA3pro</t>
+  </si>
+  <si>
+    <t>VA5pro</t>
   </si>
 </sst>
 </file>
@@ -789,42 +789,7 @@
   </cellStyleXfs>
   <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -832,9 +797,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -928,12 +890,50 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1284,6 +1284,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000001-8440-4BD7-B0A9-D8693E9D4F6B}"/>
                 </c:ext>
@@ -1312,6 +1313,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000003-8440-4BD7-B0A9-D8693E9D4F6B}"/>
                 </c:ext>
@@ -1340,6 +1342,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000005-8440-4BD7-B0A9-D8693E9D4F6B}"/>
                 </c:ext>
@@ -1368,6 +1371,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000007-8440-4BD7-B0A9-D8693E9D4F6B}"/>
                 </c:ext>
@@ -1396,6 +1400,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000009-8440-4BD7-B0A9-D8693E9D4F6B}"/>
                 </c:ext>
@@ -1424,6 +1429,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{0000000B-8440-4BD7-B0A9-D8693E9D4F6B}"/>
                 </c:ext>
@@ -1452,6 +1458,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{0000000D-8440-4BD7-B0A9-D8693E9D4F6B}"/>
                 </c:ext>
@@ -1480,6 +1487,7 @@
               <c:showPercent val="0"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{0000000F-8440-4BD7-B0A9-D8693E9D4F6B}"/>
                 </c:ext>
@@ -2012,6 +2020,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000001-7753-43DC-8986-EF7F896D4CB4}"/>
                 </c:ext>
@@ -2044,6 +2053,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000003-7753-43DC-8986-EF7F896D4CB4}"/>
                 </c:ext>
@@ -2076,6 +2086,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000005-7753-43DC-8986-EF7F896D4CB4}"/>
                 </c:ext>
@@ -2108,6 +2119,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000007-7753-43DC-8986-EF7F896D4CB4}"/>
                 </c:ext>
@@ -2140,6 +2152,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000009-7753-43DC-8986-EF7F896D4CB4}"/>
                 </c:ext>
@@ -2172,6 +2185,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{0000000B-7753-43DC-8986-EF7F896D4CB4}"/>
                 </c:ext>
@@ -2204,6 +2218,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{0000000D-7753-43DC-8986-EF7F896D4CB4}"/>
                 </c:ext>
@@ -2236,6 +2251,7 @@
               <c:showPercent val="1"/>
               <c:showBubbleSize val="1"/>
               <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{0000000F-7753-43DC-8986-EF7F896D4CB4}"/>
                 </c:ext>
@@ -3201,482 +3217,512 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
     </row>
     <row r="3" spans="2:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
     </row>
     <row r="5" spans="2:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
     </row>
     <row r="6" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="11" t="s">
+      <c r="C6" s="3"/>
+      <c r="D6" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="11"/>
+      <c r="E6" s="39"/>
     </row>
     <row r="7" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="11" t="s">
+      <c r="C7" s="3"/>
+      <c r="D7" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="11"/>
+      <c r="E7" s="39"/>
     </row>
     <row r="8" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="11" t="s">
+      <c r="C8" s="3"/>
+      <c r="D8" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="11"/>
+      <c r="E8" s="39"/>
     </row>
     <row r="9" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="11" t="s">
+      <c r="C9" s="3"/>
+      <c r="D9" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="11"/>
+      <c r="E9" s="39"/>
     </row>
     <row r="10" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="11" t="s">
+      <c r="C10" s="3"/>
+      <c r="D10" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="11"/>
+      <c r="E10" s="39"/>
     </row>
     <row r="11" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="11" t="s">
+      <c r="C11" s="3"/>
+      <c r="D11" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="11"/>
+      <c r="E11" s="39"/>
     </row>
     <row r="13" spans="2:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="42"/>
     </row>
     <row r="14" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="15" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="D15" s="6">
+        <v>21000000</v>
+      </c>
+      <c r="E15" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="20">
+    </row>
+    <row r="16" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B16" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="6">
+        <v>68000000</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="23.25" x14ac:dyDescent="0.45">
+      <c r="B17" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" s="6">
+        <v>115000000</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B19" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="19.7" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="8">
+        <f>IF(C19="VibrioM",21000000,IF(C19="VA3Pro",68000000,IF(C19="VA5pro",115000000,0)))</f>
         <v>21000000</v>
       </c>
-      <c r="E15" s="21" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="16" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="20">
-        <v>68000000</v>
-      </c>
-      <c r="E16" s="21" t="s">
+      <c r="D20" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" s="39"/>
+    </row>
+    <row r="21" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B21" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="10"/>
+      <c r="D21" s="39" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21" s="39"/>
+    </row>
+    <row r="23" spans="2:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B23" s="42" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="42"/>
+      <c r="D23" s="42"/>
+      <c r="E23" s="42"/>
+    </row>
+    <row r="24" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B24" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" s="11">
+        <v>120</v>
+      </c>
+      <c r="D24" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24" s="39"/>
+    </row>
+    <row r="25" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B25" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C25" s="11">
         <v>25</v>
       </c>
-    </row>
-    <row r="17" spans="2:5" ht="23.25" x14ac:dyDescent="0.45">
-      <c r="B17" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D17" s="20">
-        <v>115000000</v>
-      </c>
-      <c r="E17" s="21" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B19" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="16" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20" spans="2:5" ht="19.7" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C20" s="22">
-        <f>IF(C19="Vidrio",21000000,IF(C19="Ba 3 Pro",68000000,IF(C19="Ba 5",115000000,0)))</f>
-        <v>68000000</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="E20" s="11"/>
-    </row>
-    <row r="21" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E21" s="11"/>
-    </row>
-    <row r="23" spans="2:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B23" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-    </row>
-    <row r="24" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B24" s="23" t="s">
+      <c r="D25" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="25">
-        <v>120</v>
-      </c>
-      <c r="D24" s="11" t="s">
+      <c r="E25" s="39"/>
+    </row>
+    <row r="26" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B26" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="E24" s="11"/>
-    </row>
-    <row r="25" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B25" s="23" t="s">
+      <c r="C26" s="10">
+        <v>5000000</v>
+      </c>
+      <c r="D26" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="25">
-        <v>25</v>
-      </c>
-      <c r="D25" s="11" t="s">
+      <c r="E26" s="39"/>
+    </row>
+    <row r="27" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B27" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="E25" s="11"/>
-    </row>
-    <row r="26" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B26" s="23" t="s">
+      <c r="C27" s="11">
+        <v>8</v>
+      </c>
+      <c r="D27" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="24">
-        <v>5000000</v>
-      </c>
-      <c r="D26" s="11" t="s">
+      <c r="E27" s="39"/>
+    </row>
+    <row r="28" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B28" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E26" s="11"/>
-    </row>
-    <row r="27" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B27" s="23" t="s">
+      <c r="C28" s="12">
+        <v>12</v>
+      </c>
+      <c r="D28" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="25">
-        <v>8</v>
-      </c>
-      <c r="D27" s="11" t="s">
+      <c r="E28" s="39"/>
+    </row>
+    <row r="29" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B29" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E27" s="11"/>
-    </row>
-    <row r="28" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B28" s="23" t="s">
+      <c r="C29" s="10">
+        <v>15000000</v>
+      </c>
+      <c r="D29" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="C28" s="26">
-        <v>12</v>
-      </c>
-      <c r="D28" s="11" t="s">
+      <c r="E29" s="39"/>
+    </row>
+    <row r="30" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B30" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E28" s="11"/>
-    </row>
-    <row r="29" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B29" s="23" t="s">
+      <c r="C30" s="11">
+        <v>6</v>
+      </c>
+      <c r="D30" s="39" t="s">
         <v>45</v>
       </c>
-      <c r="C29" s="24">
-        <v>15000000</v>
-      </c>
-      <c r="D29" s="11" t="s">
+      <c r="E30" s="39"/>
+    </row>
+    <row r="31" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B31" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="11"/>
-    </row>
-    <row r="30" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B30" s="23" t="s">
+      <c r="C31" s="11">
+        <v>160</v>
+      </c>
+      <c r="D31" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="25">
-        <v>6</v>
-      </c>
-      <c r="D30" s="11" t="s">
+      <c r="E31" s="39"/>
+    </row>
+    <row r="32" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B32" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E30" s="11"/>
-    </row>
-    <row r="31" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B31" s="23" t="s">
+      <c r="C32" s="10">
+        <v>35000</v>
+      </c>
+      <c r="D32" s="39" t="s">
         <v>49</v>
       </c>
-      <c r="C31" s="25">
-        <v>160</v>
-      </c>
-      <c r="D31" s="11" t="s">
+      <c r="E32" s="39"/>
+    </row>
+    <row r="33" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B33" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E31" s="11"/>
-    </row>
-    <row r="32" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B32" s="23" t="s">
+      <c r="C33" s="11">
+        <v>15</v>
+      </c>
+      <c r="D33" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="C32" s="24">
-        <v>35000</v>
-      </c>
-      <c r="D32" s="11" t="s">
+      <c r="E33" s="39"/>
+    </row>
+    <row r="34" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B34" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E32" s="11"/>
-    </row>
-    <row r="33" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B33" s="23" t="s">
+      <c r="C34" s="10">
+        <v>80000000</v>
+      </c>
+      <c r="D34" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="C33" s="25">
-        <v>15</v>
-      </c>
-      <c r="D33" s="11" t="s">
+      <c r="E34" s="39"/>
+    </row>
+    <row r="35" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B35" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="E33" s="11"/>
-    </row>
-    <row r="34" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B34" s="23" t="s">
+      <c r="C35" s="11">
+        <v>200</v>
+      </c>
+      <c r="D35" s="39" t="s">
         <v>55</v>
       </c>
-      <c r="C34" s="24">
-        <v>80000000</v>
-      </c>
-      <c r="D34" s="11" t="s">
+      <c r="E35" s="39"/>
+    </row>
+    <row r="36" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B36" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E34" s="11"/>
-    </row>
-    <row r="35" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B35" s="23" t="s">
+      <c r="C36" s="10">
+        <v>2000000</v>
+      </c>
+      <c r="D36" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="C35" s="25">
-        <v>200</v>
-      </c>
-      <c r="D35" s="11" t="s">
+      <c r="E36" s="39"/>
+    </row>
+    <row r="37" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B37" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="E35" s="11"/>
-    </row>
-    <row r="36" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B36" s="23" t="s">
+      <c r="C37" s="10">
+        <v>500000000</v>
+      </c>
+      <c r="D37" s="39" t="s">
         <v>59</v>
       </c>
-      <c r="C36" s="24">
-        <v>2000000</v>
-      </c>
-      <c r="D36" s="11" t="s">
+      <c r="E37" s="39"/>
+    </row>
+    <row r="39" spans="2:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B39" s="42" t="s">
         <v>60</v>
       </c>
-      <c r="E36" s="11"/>
-    </row>
-    <row r="37" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B37" s="23" t="s">
+      <c r="C39" s="42"/>
+      <c r="D39" s="42"/>
+      <c r="E39" s="42"/>
+    </row>
+    <row r="40" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B40" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="C37" s="24">
-        <v>500000000</v>
-      </c>
-      <c r="D37" s="11" t="s">
+      <c r="C40" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="D40" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="E37" s="11"/>
-    </row>
-    <row r="39" spans="2:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B39" s="12" t="s">
+      <c r="E40" s="39"/>
+    </row>
+    <row r="41" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B41" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C39" s="12"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="12"/>
-    </row>
-    <row r="40" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B40" s="23" t="s">
+      <c r="C41" s="13">
+        <v>0.4</v>
+      </c>
+      <c r="D41" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="C40" s="27">
-        <v>0.5</v>
-      </c>
-      <c r="D40" s="11" t="s">
+      <c r="E41" s="39"/>
+    </row>
+    <row r="42" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B42" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="E40" s="11"/>
-    </row>
-    <row r="41" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B41" s="23" t="s">
+      <c r="C42" s="13">
+        <v>0.35</v>
+      </c>
+      <c r="D42" s="39" t="s">
         <v>66</v>
       </c>
-      <c r="C41" s="27">
-        <v>0.4</v>
-      </c>
-      <c r="D41" s="11" t="s">
+      <c r="E42" s="39"/>
+    </row>
+    <row r="43" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B43" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="E41" s="11"/>
-    </row>
-    <row r="42" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B42" s="23" t="s">
+      <c r="C43" s="13">
+        <v>0.25</v>
+      </c>
+      <c r="D43" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="C42" s="27">
-        <v>0.35</v>
-      </c>
-      <c r="D42" s="11" t="s">
+      <c r="E43" s="39"/>
+    </row>
+    <row r="44" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B44" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="E42" s="11"/>
-    </row>
-    <row r="43" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B43" s="23" t="s">
+      <c r="C44" s="13">
+        <v>0.2</v>
+      </c>
+      <c r="D44" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="C43" s="27">
+      <c r="E44" s="39"/>
+    </row>
+    <row r="45" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B45" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C45" s="13">
         <v>0.25</v>
       </c>
-      <c r="D43" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="E43" s="11"/>
-    </row>
-    <row r="44" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B44" s="23" t="s">
+      <c r="D45" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="C44" s="27">
-        <v>0.2</v>
-      </c>
-      <c r="D44" s="11" t="s">
+      <c r="E45" s="39"/>
+    </row>
+    <row r="46" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B46" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="E44" s="11"/>
-    </row>
-    <row r="45" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B45" s="23" t="s">
+      <c r="C46" s="13">
+        <v>0.05</v>
+      </c>
+      <c r="D46" s="39" t="s">
         <v>74</v>
       </c>
-      <c r="C45" s="27">
-        <v>0.25</v>
-      </c>
-      <c r="D45" s="11" t="s">
+      <c r="E46" s="39"/>
+    </row>
+    <row r="47" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B47" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="E45" s="11"/>
-    </row>
-    <row r="46" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B46" s="23" t="s">
+      <c r="C47" s="13">
+        <v>0.1</v>
+      </c>
+      <c r="D47" s="39" t="s">
         <v>76</v>
       </c>
-      <c r="C46" s="27">
-        <v>0.05</v>
-      </c>
-      <c r="D46" s="11" t="s">
+      <c r="E47" s="39"/>
+    </row>
+    <row r="49" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B49" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="E46" s="11"/>
-    </row>
-    <row r="47" spans="2:5" ht="28.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B47" s="23" t="s">
+      <c r="C49" s="40"/>
+      <c r="D49" s="40"/>
+      <c r="E49" s="40"/>
+    </row>
+    <row r="50" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B50" s="41" t="s">
         <v>78</v>
       </c>
-      <c r="C47" s="27">
-        <v>0.1</v>
-      </c>
-      <c r="D47" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="E47" s="11"/>
-    </row>
-    <row r="49" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B49" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="C49" s="10"/>
-      <c r="D49" s="10"/>
-      <c r="E49" s="10"/>
-    </row>
-    <row r="50" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B50" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="C50" s="9"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="9"/>
+      <c r="C50" s="41"/>
+      <c r="D50" s="41"/>
+      <c r="E50" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
     <mergeCell ref="D47:E47"/>
     <mergeCell ref="B49:E49"/>
     <mergeCell ref="B50:E50"/>
@@ -3685,36 +3731,6 @@
     <mergeCell ref="D44:E44"/>
     <mergeCell ref="D45:E45"/>
     <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" errorTitle="Modelo inválido" error="Seleccione un modelo válido" promptTitle="Modelo" prompt="Seleccione el modelo del colector" sqref="C19" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -3741,762 +3757,767 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="43" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+    </row>
+    <row r="4" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B4" s="42" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+    </row>
+    <row r="5" spans="2:7" ht="21" x14ac:dyDescent="0.45">
+      <c r="B5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="14">
+        <f>IF('Entrada de Datos'!C21&gt;0,'Entrada de Datos'!C21,'Entrada de Datos'!C20)</f>
+        <v>21000000</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B7" s="42" t="s">
+        <v>81</v>
+      </c>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="42"/>
+    </row>
+    <row r="8" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B8" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-    </row>
-    <row r="4" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="12" t="s">
+      <c r="C8" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-    </row>
-    <row r="5" spans="2:7" ht="21" x14ac:dyDescent="0.45">
-      <c r="B5" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="28">
-        <f>IF('Entrada de Datos'!C21&gt;0,'Entrada de Datos'!C21,'Entrada de Datos'!C20)</f>
-        <v>68000000</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="12" t="s">
+      <c r="D8" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-    </row>
-    <row r="8" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B8" s="17" t="s">
+      <c r="E8" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="F8" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D8" s="17" t="s">
+    </row>
+    <row r="9" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B9" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="E8" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="F8" s="17" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B9" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="C9" s="29">
+      <c r="C9" s="15">
         <f>'Entrada de Datos'!C27*'Entrada de Datos'!C28</f>
         <v>96</v>
       </c>
-      <c r="D9" s="30" t="s">
-        <v>91</v>
-      </c>
-      <c r="E9" s="29">
+      <c r="D9" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="E9" s="15">
         <f>C9*(1-'Entrada de Datos'!C40)</f>
         <v>48</v>
       </c>
-      <c r="F9" s="31">
+      <c r="F9" s="17">
         <f>C9-E9</f>
         <v>48</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B10" s="23" t="s">
-        <v>92</v>
-      </c>
-      <c r="C10" s="32">
+      <c r="B10" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" s="18">
         <f>C9*'Entrada de Datos'!C26</f>
         <v>480000000</v>
       </c>
-      <c r="D10" s="30" t="s">
-        <v>93</v>
-      </c>
-      <c r="E10" s="32">
+      <c r="D10" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E10" s="18">
         <f>E9*'Entrada de Datos'!C26</f>
         <v>240000000</v>
       </c>
-      <c r="F10" s="33">
+      <c r="F10" s="19">
         <f>C10-E10</f>
         <v>240000000</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
+      <c r="B12" s="42" t="s">
+        <v>91</v>
+      </c>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="42"/>
     </row>
     <row r="13" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="F13" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D13" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="E13" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="F13" s="17" t="s">
-        <v>89</v>
-      </c>
     </row>
     <row r="14" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B14" s="23" t="s">
-        <v>95</v>
-      </c>
-      <c r="C14" s="32">
+      <c r="B14" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="C14" s="18">
         <f>'Entrada de Datos'!C29*'Entrada de Datos'!C30</f>
         <v>90000000</v>
       </c>
-      <c r="D14" s="30" t="s">
-        <v>96</v>
-      </c>
-      <c r="E14" s="32">
+      <c r="D14" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="E14" s="18">
         <f>C14*(1-'Entrada de Datos'!C41)</f>
         <v>54000000</v>
       </c>
-      <c r="F14" s="33">
+      <c r="F14" s="19">
         <f>C14-E14</f>
         <v>36000000</v>
       </c>
     </row>
     <row r="16" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
+      <c r="B16" s="42" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="42"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="42"/>
+      <c r="F16" s="42"/>
+      <c r="G16" s="42"/>
     </row>
     <row r="17" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="F17" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D17" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="E17" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="F17" s="17" t="s">
-        <v>89</v>
-      </c>
     </row>
     <row r="18" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B18" s="23" t="s">
-        <v>98</v>
-      </c>
-      <c r="C18" s="32">
+      <c r="B18" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="C18" s="18">
         <f>'Entrada de Datos'!C31*12*'Entrada de Datos'!C32</f>
         <v>67200000</v>
       </c>
-      <c r="D18" s="30" t="s">
-        <v>99</v>
-      </c>
-      <c r="E18" s="32">
+      <c r="D18" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E18" s="18">
         <f>C18*(1-'Entrada de Datos'!C42)</f>
         <v>43680000</v>
       </c>
-      <c r="F18" s="33">
+      <c r="F18" s="19">
         <f>C18-E18</f>
         <v>23520000</v>
       </c>
     </row>
     <row r="20" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
+      <c r="B20" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="C20" s="42"/>
+      <c r="D20" s="42"/>
+      <c r="E20" s="42"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="42"/>
     </row>
     <row r="21" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C21" s="17" t="s">
+      <c r="F21" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D21" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="E21" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="F21" s="17" t="s">
-        <v>89</v>
-      </c>
     </row>
     <row r="22" spans="2:7" ht="23.25" x14ac:dyDescent="0.45">
-      <c r="B22" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="C22" s="32">
+      <c r="B22" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="18">
         <f>'Entrada de Datos'!C33*8*'Entrada de Datos'!C26*('Entrada de Datos'!C27*0.3)+'Entrada de Datos'!C34</f>
         <v>1520000000</v>
       </c>
-      <c r="D22" s="34" t="s">
-        <v>102</v>
-      </c>
-      <c r="E22" s="32">
+      <c r="D22" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="E22" s="18">
         <f>C22*(1-'Entrada de Datos'!C43)</f>
         <v>1140000000</v>
       </c>
-      <c r="F22" s="33">
+      <c r="F22" s="19">
         <f>C22-E22</f>
         <v>380000000</v>
       </c>
     </row>
     <row r="24" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B24" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-      <c r="G24" s="12"/>
+      <c r="B24" s="42" t="s">
+        <v>100</v>
+      </c>
+      <c r="C24" s="42"/>
+      <c r="D24" s="42"/>
+      <c r="E24" s="42"/>
+      <c r="F24" s="42"/>
+      <c r="G24" s="42"/>
     </row>
     <row r="25" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="F25" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D25" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="E25" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="F25" s="17" t="s">
-        <v>89</v>
-      </c>
     </row>
     <row r="26" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B26" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="C26" s="32">
+      <c r="B26" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C26" s="18">
         <f>'Entrada de Datos'!C35*'Entrada de Datos'!C36</f>
         <v>400000000</v>
       </c>
-      <c r="D26" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="E26" s="32">
+      <c r="D26" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="E26" s="18">
         <f>C26*(1-'Entrada de Datos'!C44)</f>
         <v>320000000</v>
       </c>
-      <c r="F26" s="33">
+      <c r="F26" s="19">
         <f>C26-E26</f>
         <v>80000000</v>
       </c>
     </row>
     <row r="28" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B28" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12"/>
+      <c r="B28" s="42" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" s="42"/>
+      <c r="D28" s="42"/>
+      <c r="E28" s="42"/>
+      <c r="F28" s="42"/>
+      <c r="G28" s="42"/>
     </row>
     <row r="29" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="F29" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D29" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="E29" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="F29" s="17" t="s">
-        <v>89</v>
-      </c>
     </row>
     <row r="30" spans="2:7" ht="23.25" x14ac:dyDescent="0.45">
-      <c r="B30" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="C30" s="32">
+      <c r="B30" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C30" s="18">
         <f>'Entrada de Datos'!C25*50000000/15</f>
         <v>83333333.333333328</v>
       </c>
-      <c r="D30" s="34" t="s">
-        <v>108</v>
-      </c>
-      <c r="E30" s="35">
+      <c r="D30" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="E30" s="21">
         <f>C30</f>
         <v>83333333.333333328</v>
       </c>
-      <c r="F30" s="33">
+      <c r="F30" s="19">
         <f>C30*'Entrada de Datos'!C45</f>
         <v>20833333.333333332</v>
       </c>
     </row>
     <row r="32" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B32" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
+      <c r="B32" s="42" t="s">
+        <v>106</v>
+      </c>
+      <c r="C32" s="42"/>
+      <c r="D32" s="42"/>
+      <c r="E32" s="42"/>
+      <c r="F32" s="42"/>
+      <c r="G32" s="42"/>
     </row>
     <row r="33" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E33" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C33" s="17" t="s">
+      <c r="F33" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D33" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="E33" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="F33" s="17" t="s">
-        <v>89</v>
-      </c>
     </row>
     <row r="34" spans="2:7" ht="23.25" x14ac:dyDescent="0.45">
-      <c r="B34" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="C34" s="32">
+      <c r="B34" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C34" s="18">
         <f>'Entrada de Datos'!C24*50*0.746*6000*500</f>
         <v>13428000000</v>
       </c>
-      <c r="D34" s="34" t="s">
-        <v>111</v>
-      </c>
-      <c r="E34" s="32">
+      <c r="D34" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="E34" s="18">
         <f>C34</f>
         <v>13428000000</v>
       </c>
-      <c r="F34" s="33">
+      <c r="F34" s="19">
         <f>C34*'Entrada de Datos'!C46</f>
         <v>671400000</v>
       </c>
     </row>
     <row r="36" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B36" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="C36" s="12"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
-      <c r="G36" s="12"/>
+      <c r="B36" s="42" t="s">
+        <v>109</v>
+      </c>
+      <c r="C36" s="42"/>
+      <c r="D36" s="42"/>
+      <c r="E36" s="42"/>
+      <c r="F36" s="42"/>
+      <c r="G36" s="42"/>
     </row>
     <row r="37" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B37" s="17" t="s">
+      <c r="B37" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E37" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C37" s="17" t="s">
+      <c r="F37" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D37" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="E37" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="F37" s="17" t="s">
-        <v>89</v>
-      </c>
     </row>
     <row r="38" spans="2:7" ht="23.25" x14ac:dyDescent="0.45">
-      <c r="B38" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="C38" s="32">
+      <c r="B38" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="C38" s="18">
         <f>'Entrada de Datos'!C37*12*0.02</f>
         <v>120000000</v>
       </c>
-      <c r="D38" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="E38" s="32">
+      <c r="D38" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="E38" s="18">
         <f>C38</f>
         <v>120000000</v>
       </c>
-      <c r="F38" s="33">
+      <c r="F38" s="19">
         <f>C38*'Entrada de Datos'!C47</f>
         <v>12000000</v>
       </c>
     </row>
     <row r="40" spans="2:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B40" s="14" t="s">
+      <c r="B40" s="43" t="s">
+        <v>112</v>
+      </c>
+      <c r="C40" s="43"/>
+      <c r="D40" s="43"/>
+      <c r="E40" s="43"/>
+      <c r="F40" s="43"/>
+      <c r="G40" s="43"/>
+    </row>
+    <row r="42" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B42" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-    </row>
-    <row r="42" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B42" s="17" t="s">
+    </row>
+    <row r="43" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B43" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="C42" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="D42" s="17" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="43" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B43" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="C43" s="36">
+      <c r="C43" s="22">
         <f>F10</f>
         <v>240000000</v>
       </c>
-      <c r="D43" s="37">
+      <c r="D43" s="23">
         <f>IF(C51&gt;0,C43/C51,0)</f>
         <v>0.16396205189398941</v>
       </c>
     </row>
     <row r="44" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B44" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="C44" s="36">
+      <c r="B44" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="C44" s="22">
         <f>F14</f>
         <v>36000000</v>
       </c>
-      <c r="D44" s="37">
+      <c r="D44" s="23">
         <f>IF(C51&gt;0,C44/C51,0)</f>
         <v>2.459430778409841E-2</v>
       </c>
     </row>
     <row r="45" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B45" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="C45" s="36">
+      <c r="B45" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="C45" s="22">
         <f>F18</f>
         <v>23520000</v>
       </c>
-      <c r="D45" s="37">
+      <c r="D45" s="23">
         <f>IF(C51&gt;0,C45/C51,0)</f>
         <v>1.6068281085610963E-2</v>
       </c>
     </row>
     <row r="46" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B46" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="C46" s="36">
+      <c r="B46" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C46" s="22">
         <f>F22</f>
         <v>380000000</v>
       </c>
-      <c r="D46" s="37">
+      <c r="D46" s="23">
         <f>IF(C51&gt;0,C46/C51,0)</f>
         <v>0.25960658216548321</v>
       </c>
     </row>
     <row r="47" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B47" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="C47" s="36">
+      <c r="B47" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="C47" s="22">
         <f>F26</f>
         <v>80000000</v>
       </c>
-      <c r="D47" s="37">
+      <c r="D47" s="23">
         <f>IF(C51&gt;0,C47/C51,0)</f>
         <v>5.4654017297996467E-2</v>
       </c>
     </row>
     <row r="48" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B48" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="C48" s="36">
+      <c r="B48" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="C48" s="22">
         <f>F30</f>
         <v>20833333.333333332</v>
       </c>
-      <c r="D48" s="37">
+      <c r="D48" s="23">
         <f>IF(C51&gt;0,C48/C51,0)</f>
         <v>1.4232817004686579E-2</v>
       </c>
     </row>
     <row r="49" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B49" s="23" t="s">
-        <v>125</v>
-      </c>
-      <c r="C49" s="36">
+      <c r="B49" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="C49" s="22">
         <f>F34</f>
         <v>671400000</v>
       </c>
-      <c r="D49" s="37">
+      <c r="D49" s="23">
         <f>IF(C51&gt;0,C49/C51,0)</f>
         <v>0.45868384017343539</v>
       </c>
     </row>
     <row r="50" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B50" s="23" t="s">
-        <v>126</v>
-      </c>
-      <c r="C50" s="36">
+      <c r="B50" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="C50" s="22">
         <f>F38</f>
         <v>12000000</v>
       </c>
-      <c r="D50" s="37">
+      <c r="D50" s="23">
         <f>IF(C51&gt;0,C50/C51,0)</f>
         <v>8.1981025946994707E-3</v>
       </c>
     </row>
     <row r="51" spans="2:7" ht="18" x14ac:dyDescent="0.45">
-      <c r="B51" s="38" t="s">
-        <v>127</v>
-      </c>
-      <c r="C51" s="39">
+      <c r="B51" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="C51" s="25">
         <f>SUM(C43:C50)</f>
         <v>1463753333.3333335</v>
       </c>
-      <c r="D51" s="40" t="s">
-        <v>128</v>
+      <c r="D51" s="26" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="53" spans="2:7" ht="21" x14ac:dyDescent="0.45">
-      <c r="B53" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="C53" s="28">
+      <c r="B53" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C53" s="14">
         <f>C5</f>
-        <v>68000000</v>
+        <v>21000000</v>
       </c>
     </row>
     <row r="54" spans="2:7" ht="18" x14ac:dyDescent="0.45">
-      <c r="B54" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="C54" s="41">
+      <c r="B54" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C54" s="27">
         <f>C51</f>
         <v>1463753333.3333335</v>
       </c>
     </row>
     <row r="55" spans="2:7" ht="21" x14ac:dyDescent="0.45">
-      <c r="B55" s="15" t="s">
+      <c r="B55" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C55" s="28">
+        <f>IF(C53&gt;0,(C54-C53)/C53,0)</f>
+        <v>68.702539682539694</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" ht="21" x14ac:dyDescent="0.45">
+      <c r="B56" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C56" s="29">
+        <f>IF(C54&gt;0,ROUND(C53/(C54/12),1),"N/A")</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="57" spans="2:7" ht="21" x14ac:dyDescent="0.45">
+      <c r="B57" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C57" s="30">
+        <f>IF(C53&gt;0,C54/C53,0)</f>
+        <v>69.702539682539694</v>
+      </c>
+    </row>
+    <row r="59" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B59" s="42" t="s">
         <v>131</v>
       </c>
-      <c r="C55" s="42">
-        <f>IF(C53&gt;0,(C54-C53)/C53,0)</f>
-        <v>20.525784313725492</v>
-      </c>
-    </row>
-    <row r="56" spans="2:7" ht="21" x14ac:dyDescent="0.45">
-      <c r="B56" s="15" t="s">
+      <c r="C59" s="42"/>
+      <c r="D59" s="42"/>
+      <c r="E59" s="42"/>
+      <c r="F59" s="42"/>
+      <c r="G59" s="42"/>
+    </row>
+    <row r="60" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B60" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C60" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="C56" s="43">
-        <f>IF(C54&gt;0,ROUND(C53/(C54/12),1),"N/A")</f>
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="57" spans="2:7" ht="21" x14ac:dyDescent="0.45">
-      <c r="B57" s="15" t="s">
+      <c r="D60" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C57" s="44">
-        <f>IF(C53&gt;0,C54/C53,0)</f>
-        <v>21.525784313725492</v>
-      </c>
-    </row>
-    <row r="59" spans="2:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B59" s="12" t="s">
+      <c r="E60" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C59" s="12"/>
-      <c r="D59" s="12"/>
-      <c r="E59" s="12"/>
-      <c r="F59" s="12"/>
-      <c r="G59" s="12"/>
-    </row>
-    <row r="60" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B60" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="C60" s="17" t="s">
+      <c r="F60" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D60" s="17" t="s">
+      <c r="G60" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E60" s="17" t="s">
+    </row>
+    <row r="61" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B61" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="F60" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="G60" s="17" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="61" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B61" s="23" t="s">
-        <v>140</v>
-      </c>
-      <c r="C61" s="36">
+      <c r="C61" s="22">
         <f>C51</f>
         <v>1463753333.3333335</v>
       </c>
-      <c r="D61" s="36">
+      <c r="D61" s="22">
         <f>C51</f>
         <v>1463753333.3333335</v>
       </c>
-      <c r="E61" s="36">
+      <c r="E61" s="22">
         <f>C51</f>
         <v>1463753333.3333335</v>
       </c>
-      <c r="F61" s="36">
+      <c r="F61" s="22">
         <f>C51</f>
         <v>1463753333.3333335</v>
       </c>
-      <c r="G61" s="36">
+      <c r="G61" s="22">
         <f>C51</f>
         <v>1463753333.3333335</v>
       </c>
     </row>
     <row r="62" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B62" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="C62" s="36">
+      <c r="B62" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="C62" s="22">
         <f>C61</f>
         <v>1463753333.3333335</v>
       </c>
-      <c r="D62" s="36">
+      <c r="D62" s="22">
         <f>C62+D61</f>
         <v>2927506666.666667</v>
       </c>
-      <c r="E62" s="36">
+      <c r="E62" s="22">
         <f>D62+E61</f>
         <v>4391260000</v>
       </c>
-      <c r="F62" s="36">
+      <c r="F62" s="22">
         <f>E62+F61</f>
         <v>5855013333.333334</v>
       </c>
-      <c r="G62" s="36">
+      <c r="G62" s="22">
         <f>F62+G61</f>
         <v>7318766666.6666679</v>
       </c>
     </row>
     <row r="63" spans="2:7" ht="18" x14ac:dyDescent="0.45">
-      <c r="B63" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="C63" s="45">
+      <c r="B63" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="C63" s="31">
         <f>C5</f>
-        <v>68000000</v>
-      </c>
-      <c r="D63" s="36">
+        <v>21000000</v>
+      </c>
+      <c r="D63" s="22">
         <v>0</v>
       </c>
-      <c r="E63" s="36">
+      <c r="E63" s="22">
         <v>0</v>
       </c>
-      <c r="F63" s="36">
+      <c r="F63" s="22">
         <v>0</v>
       </c>
-      <c r="G63" s="36">
+      <c r="G63" s="22">
         <v>0</v>
       </c>
     </row>
     <row r="64" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B64" s="23" t="s">
-        <v>143</v>
-      </c>
-      <c r="C64" s="46">
+      <c r="B64" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="C64" s="32">
         <f>C62-C63</f>
-        <v>1395753333.3333335</v>
-      </c>
-      <c r="D64" s="46">
+        <v>1442753333.3333335</v>
+      </c>
+      <c r="D64" s="32">
         <f>D62-C63</f>
-        <v>2859506666.666667</v>
-      </c>
-      <c r="E64" s="46">
+        <v>2906506666.666667</v>
+      </c>
+      <c r="E64" s="32">
         <f>E62-C63</f>
-        <v>4323260000</v>
-      </c>
-      <c r="F64" s="46">
+        <v>4370260000</v>
+      </c>
+      <c r="F64" s="32">
         <f>F62-C63</f>
-        <v>5787013333.333334</v>
-      </c>
-      <c r="G64" s="46">
+        <v>5834013333.333334</v>
+      </c>
+      <c r="G64" s="32">
         <f>G62-C63</f>
-        <v>7250766666.6666679</v>
+        <v>7297766666.6666679</v>
       </c>
     </row>
     <row r="65" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B65" s="23" t="s">
-        <v>144</v>
-      </c>
-      <c r="C65" s="47">
+      <c r="B65" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="C65" s="33">
         <f>IF(C63&gt;0,C64/C63,0)</f>
-        <v>20.525784313725492</v>
-      </c>
-      <c r="D65" s="47">
+        <v>68.702539682539694</v>
+      </c>
+      <c r="D65" s="33">
         <f>IF(C63&gt;0,D64/C63,0)</f>
-        <v>42.051568627450983</v>
-      </c>
-      <c r="E65" s="47">
+        <v>138.40507936507939</v>
+      </c>
+      <c r="E65" s="33">
         <f>IF(C63&gt;0,E64/C63,0)</f>
-        <v>63.577352941176471</v>
-      </c>
-      <c r="F65" s="47">
+        <v>208.10761904761904</v>
+      </c>
+      <c r="F65" s="33">
         <f>IF(C63&gt;0,F64/C63,0)</f>
-        <v>85.103137254901966</v>
-      </c>
-      <c r="G65" s="47">
+        <v>277.81015873015878</v>
+      </c>
+      <c r="G65" s="33">
         <f>IF(C63&gt;0,G64/C63,0)</f>
-        <v>106.62892156862748</v>
+        <v>347.51269841269846</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B16:G16"/>
     <mergeCell ref="B40:G40"/>
     <mergeCell ref="B59:G59"/>
     <mergeCell ref="B20:G20"/>
@@ -4504,11 +4525,6 @@
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B32:G32"/>
     <mergeCell ref="B36:G36"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B12:G12"/>
-    <mergeCell ref="B16:G16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -4531,443 +4547,443 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="49.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="43" t="s">
+        <v>142</v>
+      </c>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+    </row>
+    <row r="3" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B3" s="54" t="s">
+        <v>143</v>
+      </c>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+    </row>
+    <row r="4" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B4" s="44" t="s">
+        <v>144</v>
+      </c>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="44"/>
+    </row>
+    <row r="6" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B6" s="55" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
+    </row>
+    <row r="7" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B7" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-    </row>
-    <row r="3" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-    </row>
-    <row r="4" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-    </row>
-    <row r="6" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-    </row>
-    <row r="7" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B7" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="C7" s="48">
+      <c r="C7" s="34">
         <f>'Entrada de Datos'!C6</f>
         <v>0</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="E7" s="48">
+      <c r="D7" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E7" s="34">
         <f>'Entrada de Datos'!C7</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B8" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="C8" s="48">
+      <c r="B8" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C8" s="34">
         <f>'Entrada de Datos'!C8</f>
         <v>0</v>
       </c>
-      <c r="D8" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="E8" s="48">
+      <c r="D8" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E8" s="34">
         <f>'Entrada de Datos'!C11</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
+      <c r="B10" s="45" t="s">
+        <v>149</v>
+      </c>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="45"/>
     </row>
     <row r="11" spans="2:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="G11" s="5"/>
+      <c r="B11" s="49" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49" t="s">
+        <v>150</v>
+      </c>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49" t="s">
+        <v>86</v>
+      </c>
+      <c r="G11" s="49"/>
     </row>
     <row r="12" spans="2:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="4" t="str">
+      <c r="B12" s="52" t="str">
         <f>'Entrada de Datos'!C19</f>
-        <v>Ba 3 Pro</v>
-      </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="3">
+        <v>VibrioM</v>
+      </c>
+      <c r="C12" s="52"/>
+      <c r="D12" s="53">
         <f>'Cálculos Internos'!C5</f>
-        <v>68000000</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="49">
+        <v>21000000</v>
+      </c>
+      <c r="E12" s="53"/>
+      <c r="F12" s="35">
         <f>'Cálculos Internos'!C51</f>
         <v>1463753333.3333335</v>
       </c>
     </row>
     <row r="13" spans="2:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="49" t="s">
+        <v>151</v>
+      </c>
+      <c r="C13" s="49"/>
+      <c r="D13" s="49" t="s">
+        <v>152</v>
+      </c>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49" t="s">
+        <v>153</v>
+      </c>
+      <c r="G13" s="49"/>
+    </row>
+    <row r="14" spans="2:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B14" s="50">
+        <f>'Cálculos Internos'!C55</f>
+        <v>68.702539682539694</v>
+      </c>
+      <c r="C14" s="50"/>
+      <c r="D14" s="51">
+        <f>'Cálculos Internos'!C56</f>
+        <v>0.2</v>
+      </c>
+      <c r="E14" s="51"/>
+      <c r="F14" s="36">
+        <f>'Cálculos Internos'!C57</f>
+        <v>69.702539682539694</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B16" s="45" t="s">
         <v>154</v>
       </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5" t="s">
+      <c r="C16" s="45"/>
+      <c r="D16" s="45"/>
+      <c r="E16" s="45"/>
+      <c r="F16" s="45"/>
+    </row>
+    <row r="17" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B17" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5" t="s">
+    </row>
+    <row r="18" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B18" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="G13" s="5"/>
-    </row>
-    <row r="14" spans="2:7" ht="34.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="2">
-        <f>'Cálculos Internos'!C55</f>
-        <v>20.525784313725492</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="1">
-        <f>'Cálculos Internos'!C56</f>
-        <v>0.6</v>
-      </c>
-      <c r="E14" s="1"/>
-      <c r="F14" s="50">
-        <f>'Cálculos Internos'!C57</f>
-        <v>21.525784313725492</v>
-      </c>
-    </row>
-    <row r="16" spans="2:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-    </row>
-    <row r="17" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B17" s="17" t="s">
-        <v>116</v>
-      </c>
-      <c r="C17" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="D17" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="E17" s="17" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="18" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B18" s="23" t="s">
-        <v>159</v>
-      </c>
-      <c r="C18" s="36">
+      <c r="C18" s="22">
         <f>'Cálculos Internos'!C43</f>
         <v>240000000</v>
       </c>
-      <c r="D18" s="37">
+      <c r="D18" s="23">
         <f>'Cálculos Internos'!D43</f>
         <v>0.16396205189398941</v>
       </c>
-      <c r="E18" s="36">
+      <c r="E18" s="22">
         <f t="shared" ref="E18:E26" si="0">C18/12</f>
         <v>20000000</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B19" s="23" t="s">
-        <v>160</v>
-      </c>
-      <c r="C19" s="36">
+      <c r="B19" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="C19" s="22">
         <f>'Cálculos Internos'!C44</f>
         <v>36000000</v>
       </c>
-      <c r="D19" s="37">
+      <c r="D19" s="23">
         <f>'Cálculos Internos'!D44</f>
         <v>2.459430778409841E-2</v>
       </c>
-      <c r="E19" s="36">
+      <c r="E19" s="22">
         <f t="shared" si="0"/>
         <v>3000000</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B20" s="23" t="s">
-        <v>161</v>
-      </c>
-      <c r="C20" s="36">
+      <c r="B20" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="C20" s="22">
         <f>'Cálculos Internos'!C45</f>
         <v>23520000</v>
       </c>
-      <c r="D20" s="37">
+      <c r="D20" s="23">
         <f>'Cálculos Internos'!D45</f>
         <v>1.6068281085610963E-2</v>
       </c>
-      <c r="E20" s="36">
+      <c r="E20" s="22">
         <f t="shared" si="0"/>
         <v>1960000</v>
       </c>
     </row>
     <row r="21" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B21" s="23" t="s">
-        <v>162</v>
-      </c>
-      <c r="C21" s="36">
+      <c r="B21" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="C21" s="22">
         <f>'Cálculos Internos'!C46</f>
         <v>380000000</v>
       </c>
-      <c r="D21" s="37">
+      <c r="D21" s="23">
         <f>'Cálculos Internos'!D46</f>
         <v>0.25960658216548321</v>
       </c>
-      <c r="E21" s="36">
+      <c r="E21" s="22">
         <f t="shared" si="0"/>
         <v>31666666.666666668</v>
       </c>
     </row>
     <row r="22" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B22" s="23" t="s">
-        <v>163</v>
-      </c>
-      <c r="C22" s="36">
+      <c r="B22" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="C22" s="22">
         <f>'Cálculos Internos'!C47</f>
         <v>80000000</v>
       </c>
-      <c r="D22" s="37">
+      <c r="D22" s="23">
         <f>'Cálculos Internos'!D47</f>
         <v>5.4654017297996467E-2</v>
       </c>
-      <c r="E22" s="36">
+      <c r="E22" s="22">
         <f t="shared" si="0"/>
         <v>6666666.666666667</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B23" s="23" t="s">
-        <v>164</v>
-      </c>
-      <c r="C23" s="36">
+      <c r="B23" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C23" s="22">
         <f>'Cálculos Internos'!C48</f>
         <v>20833333.333333332</v>
       </c>
-      <c r="D23" s="37">
+      <c r="D23" s="23">
         <f>'Cálculos Internos'!D48</f>
         <v>1.4232817004686579E-2</v>
       </c>
-      <c r="E23" s="36">
+      <c r="E23" s="22">
         <f t="shared" si="0"/>
         <v>1736111.111111111</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B24" s="23" t="s">
-        <v>165</v>
-      </c>
-      <c r="C24" s="36">
+      <c r="B24" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C24" s="22">
         <f>'Cálculos Internos'!C49</f>
         <v>671400000</v>
       </c>
-      <c r="D24" s="37">
+      <c r="D24" s="23">
         <f>'Cálculos Internos'!D49</f>
         <v>0.45868384017343539</v>
       </c>
-      <c r="E24" s="36">
+      <c r="E24" s="22">
         <f t="shared" si="0"/>
         <v>55950000</v>
       </c>
     </row>
     <row r="25" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B25" s="23" t="s">
-        <v>166</v>
-      </c>
-      <c r="C25" s="36">
+      <c r="B25" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C25" s="22">
         <f>'Cálculos Internos'!C50</f>
         <v>12000000</v>
       </c>
-      <c r="D25" s="37">
+      <c r="D25" s="23">
         <f>'Cálculos Internos'!D50</f>
         <v>8.1981025946994707E-3</v>
       </c>
-      <c r="E25" s="36">
+      <c r="E25" s="22">
         <f t="shared" si="0"/>
         <v>1000000</v>
       </c>
     </row>
     <row r="26" spans="2:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B26" s="51" t="s">
-        <v>167</v>
-      </c>
-      <c r="C26" s="52">
+      <c r="B26" s="37" t="s">
+        <v>164</v>
+      </c>
+      <c r="C26" s="38">
         <f>SUM(C18:C25)</f>
         <v>1463753333.3333335</v>
       </c>
-      <c r="D26" s="40" t="s">
-        <v>128</v>
-      </c>
-      <c r="E26" s="52">
+      <c r="D26" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="E26" s="38">
         <f t="shared" si="0"/>
         <v>121979444.44444446</v>
       </c>
     </row>
     <row r="60" spans="2:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B60" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="C60" s="6"/>
-      <c r="D60" s="6"/>
-      <c r="E60" s="6"/>
-      <c r="F60" s="6"/>
+      <c r="B60" s="45" t="s">
+        <v>165</v>
+      </c>
+      <c r="C60" s="45"/>
+      <c r="D60" s="45"/>
+      <c r="E60" s="45"/>
+      <c r="F60" s="45"/>
     </row>
     <row r="61" spans="2:7" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="B61" s="17"/>
-      <c r="C61" s="17" t="s">
+      <c r="B61" s="1"/>
+      <c r="C61" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F61" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D61" s="17" t="s">
+      <c r="G61" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E61" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="F61" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="G61" s="17" t="s">
-        <v>139</v>
-      </c>
     </row>
     <row r="62" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B62" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="C62" s="46">
+      <c r="B62" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C62" s="32">
         <f>'Cálculos Internos'!C62</f>
         <v>1463753333.3333335</v>
       </c>
-      <c r="D62" s="46">
+      <c r="D62" s="32">
         <f>'Cálculos Internos'!D62</f>
         <v>2927506666.666667</v>
       </c>
-      <c r="E62" s="46">
+      <c r="E62" s="32">
         <f>'Cálculos Internos'!E62</f>
         <v>4391260000</v>
       </c>
-      <c r="F62" s="46">
+      <c r="F62" s="32">
         <f>'Cálculos Internos'!F62</f>
         <v>5855013333.333334</v>
       </c>
-      <c r="G62" s="46">
+      <c r="G62" s="32">
         <f>'Cálculos Internos'!G62</f>
         <v>7318766666.6666679</v>
       </c>
     </row>
     <row r="63" spans="2:7" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B63" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="C63" s="36">
+      <c r="B63" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C63" s="22">
         <f>'Cálculos Internos'!C59</f>
         <v>0</v>
       </c>
-      <c r="D63" s="36">
+      <c r="D63" s="22">
         <f>'Cálculos Internos'!D59</f>
         <v>0</v>
       </c>
-      <c r="E63" s="36">
+      <c r="E63" s="22">
         <f>'Cálculos Internos'!E59</f>
         <v>0</v>
       </c>
-      <c r="F63" s="36">
+      <c r="F63" s="22">
         <f>'Cálculos Internos'!F59</f>
         <v>0</v>
       </c>
-      <c r="G63" s="36">
+      <c r="G63" s="22">
         <f>'Cálculos Internos'!G59</f>
         <v>0</v>
       </c>
     </row>
     <row r="81" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B81" s="53" t="s">
-        <v>169</v>
-      </c>
-      <c r="C81" s="53"/>
-      <c r="D81" s="53"/>
-      <c r="E81" s="53"/>
-      <c r="F81" s="53"/>
+      <c r="B81" s="46" t="s">
+        <v>166</v>
+      </c>
+      <c r="C81" s="46"/>
+      <c r="D81" s="46"/>
+      <c r="E81" s="46"/>
+      <c r="F81" s="46"/>
     </row>
     <row r="82" spans="2:6" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B82" s="54" t="s">
-        <v>170</v>
-      </c>
-      <c r="C82" s="54"/>
-      <c r="D82" s="54"/>
-      <c r="E82" s="54"/>
-      <c r="F82" s="54"/>
+      <c r="B82" s="47" t="s">
+        <v>167</v>
+      </c>
+      <c r="C82" s="47"/>
+      <c r="D82" s="47"/>
+      <c r="E82" s="47"/>
+      <c r="F82" s="47"/>
     </row>
     <row r="83" spans="2:6" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="B83" s="55" t="s">
-        <v>171</v>
-      </c>
-      <c r="C83" s="55"/>
-      <c r="D83" s="55"/>
-      <c r="E83" s="55"/>
-      <c r="F83" s="55"/>
+      <c r="B83" s="48" t="s">
+        <v>168</v>
+      </c>
+      <c r="C83" s="48"/>
+      <c r="D83" s="48"/>
+      <c r="E83" s="48"/>
+      <c r="F83" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D14:E14"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B60:F60"/>
     <mergeCell ref="B81:F81"/>
     <mergeCell ref="B82:F82"/>
     <mergeCell ref="B83:F83"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B10:F10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup fitToHeight="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>